<commit_message>
updated basetest and and other test classes
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/LoginData.xlsx
+++ b/src/main/resources/testdata/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saiku\Projects\selenium-hybrid-framework\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C87B31-8F03-4DFF-9DAF-42F35C052D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E1F455-A9A9-4CF1-8EB8-2D47C508F6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <t>problem_user</t>
   </si>
   <si>
-    <t>locked_out_user</t>
+    <t>visual_user</t>
   </si>
 </sst>
 </file>

</xml_diff>